<commit_message>
Refresh the example master sheet from the current seeded library.
Co-authored-by: hady-dotcom <hady-dotcom@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/hearts-prototype/artifacts/hearts-master-sheet-example.xlsx
+++ b/hearts-prototype/artifacts/hearts-master-sheet-example.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="995" uniqueCount="385">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1002" uniqueCount="386">
   <si>
     <t>HEARTS talks. One row is one talk. talk_key is how a later import finds the same talk, so keep it stable. Leave a cell blank to leave that field as it is. Times can be seconds (90), minutes and seconds (1:30) or hours (1:02:03). status is draft, checked or live. rejected keeps a talk hidden from learners. delete removes the talk. youtube_id is the 11-character YouTube id.</t>
   </si>
@@ -1117,6 +1117,9 @@
   </si>
   <si>
     <t>The speaker says: “Aside for loot Prophet lot for he used to certainly seek strength in the strongest corner” What does that line ask of you this week?</t>
+  </si>
+  <si>
+    <t>The speaker says: “Down repeat it recite it memorize it and it's important in fact to memorize it and teach it to others as” What does that line ask of you this week?</t>
   </si>
   <si>
     <t>The speaker says: “This powerful dua think about it” What does that line ask of you this week?</t>
@@ -3317,7 +3320,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P85"/>
+  <dimension ref="A1:P86"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="12" width="14" customWidth="1"/>
@@ -3403,7 +3406,7 @@
         <v>22</v>
       </c>
       <c r="C3">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>288</v>
@@ -3432,7 +3435,7 @@
         <v>22</v>
       </c>
       <c r="C4">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>288</v>
@@ -3461,7 +3464,7 @@
         <v>34</v>
       </c>
       <c r="C5">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>288</v>
@@ -3490,7 +3493,7 @@
         <v>34</v>
       </c>
       <c r="C6">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>288</v>
@@ -3519,7 +3522,7 @@
         <v>34</v>
       </c>
       <c r="C7">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>288</v>
@@ -3548,7 +3551,7 @@
         <v>268</v>
       </c>
       <c r="C8">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>288</v>
@@ -3577,7 +3580,7 @@
         <v>268</v>
       </c>
       <c r="C9">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D9" s="3" t="s">
         <v>288</v>
@@ -3606,7 +3609,7 @@
         <v>268</v>
       </c>
       <c r="C10">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D10" s="3" t="s">
         <v>288</v>
@@ -3635,7 +3638,7 @@
         <v>261</v>
       </c>
       <c r="C11">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D11" s="3" t="s">
         <v>288</v>
@@ -3664,7 +3667,7 @@
         <v>261</v>
       </c>
       <c r="C12">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D12" s="3" t="s">
         <v>288</v>
@@ -3693,7 +3696,7 @@
         <v>261</v>
       </c>
       <c r="C13">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D13" s="3" t="s">
         <v>288</v>
@@ -3722,7 +3725,7 @@
         <v>43</v>
       </c>
       <c r="C14">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D14" s="3" t="s">
         <v>288</v>
@@ -3751,7 +3754,7 @@
         <v>43</v>
       </c>
       <c r="C15">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D15" s="3" t="s">
         <v>288</v>
@@ -3780,7 +3783,7 @@
         <v>43</v>
       </c>
       <c r="C16">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D16" s="3" t="s">
         <v>288</v>
@@ -3809,7 +3812,7 @@
         <v>52</v>
       </c>
       <c r="C17">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D17" s="3" t="s">
         <v>288</v>
@@ -3838,7 +3841,7 @@
         <v>52</v>
       </c>
       <c r="C18">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D18" s="3" t="s">
         <v>288</v>
@@ -3867,7 +3870,7 @@
         <v>52</v>
       </c>
       <c r="C19">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D19" s="3" t="s">
         <v>288</v>
@@ -3896,7 +3899,7 @@
         <v>61</v>
       </c>
       <c r="C20">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D20" s="3" t="s">
         <v>288</v>
@@ -3925,7 +3928,7 @@
         <v>61</v>
       </c>
       <c r="C21">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D21" s="3" t="s">
         <v>288</v>
@@ -3954,7 +3957,7 @@
         <v>69</v>
       </c>
       <c r="C22">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D22" s="3" t="s">
         <v>288</v>
@@ -3983,7 +3986,7 @@
         <v>69</v>
       </c>
       <c r="C23">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D23" s="3" t="s">
         <v>288</v>
@@ -4012,7 +4015,7 @@
         <v>78</v>
       </c>
       <c r="C24">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D24" s="3" t="s">
         <v>288</v>
@@ -4041,7 +4044,7 @@
         <v>78</v>
       </c>
       <c r="C25">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D25" s="3" t="s">
         <v>288</v>
@@ -4070,7 +4073,7 @@
         <v>86</v>
       </c>
       <c r="C26">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D26" s="3" t="s">
         <v>288</v>
@@ -4099,7 +4102,7 @@
         <v>86</v>
       </c>
       <c r="C27">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D27" s="3" t="s">
         <v>288</v>
@@ -4128,7 +4131,7 @@
         <v>93</v>
       </c>
       <c r="C28">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D28" s="3" t="s">
         <v>288</v>
@@ -4157,7 +4160,7 @@
         <v>93</v>
       </c>
       <c r="C29">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D29" s="3" t="s">
         <v>288</v>
@@ -4186,7 +4189,7 @@
         <v>93</v>
       </c>
       <c r="C30">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D30" s="3" t="s">
         <v>288</v>
@@ -4215,7 +4218,7 @@
         <v>102</v>
       </c>
       <c r="C31">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D31" s="3" t="s">
         <v>288</v>
@@ -4244,7 +4247,7 @@
         <v>102</v>
       </c>
       <c r="C32">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D32" s="3" t="s">
         <v>288</v>
@@ -4273,7 +4276,7 @@
         <v>109</v>
       </c>
       <c r="C33">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D33" s="3" t="s">
         <v>288</v>
@@ -4302,7 +4305,7 @@
         <v>109</v>
       </c>
       <c r="C34">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D34" s="3" t="s">
         <v>288</v>
@@ -4331,7 +4334,7 @@
         <v>117</v>
       </c>
       <c r="C35">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D35" s="3" t="s">
         <v>288</v>
@@ -4360,7 +4363,7 @@
         <v>117</v>
       </c>
       <c r="C36">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D36" s="3" t="s">
         <v>288</v>
@@ -4389,7 +4392,7 @@
         <v>127</v>
       </c>
       <c r="C37">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D37" s="3" t="s">
         <v>288</v>
@@ -4418,7 +4421,7 @@
         <v>127</v>
       </c>
       <c r="C38">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D38" s="3" t="s">
         <v>288</v>
@@ -4447,7 +4450,7 @@
         <v>127</v>
       </c>
       <c r="C39">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D39" s="3" t="s">
         <v>288</v>
@@ -4476,7 +4479,7 @@
         <v>135</v>
       </c>
       <c r="C40">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D40" s="3" t="s">
         <v>288</v>
@@ -4505,7 +4508,7 @@
         <v>135</v>
       </c>
       <c r="C41">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D41" s="3" t="s">
         <v>288</v>
@@ -4534,7 +4537,7 @@
         <v>252</v>
       </c>
       <c r="C42">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D42" s="3" t="s">
         <v>288</v>
@@ -4563,7 +4566,7 @@
         <v>252</v>
       </c>
       <c r="C43">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D43" s="3" t="s">
         <v>288</v>
@@ -4592,7 +4595,7 @@
         <v>252</v>
       </c>
       <c r="C44">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D44" s="3" t="s">
         <v>288</v>
@@ -4621,7 +4624,7 @@
         <v>142</v>
       </c>
       <c r="C45">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D45" s="3" t="s">
         <v>288</v>
@@ -4650,7 +4653,7 @@
         <v>142</v>
       </c>
       <c r="C46">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D46" s="3" t="s">
         <v>288</v>
@@ -4679,7 +4682,7 @@
         <v>142</v>
       </c>
       <c r="C47">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D47" s="3" t="s">
         <v>288</v>
@@ -4708,7 +4711,7 @@
         <v>149</v>
       </c>
       <c r="C48">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D48" s="3" t="s">
         <v>288</v>
@@ -4737,7 +4740,7 @@
         <v>149</v>
       </c>
       <c r="C49">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D49" s="3" t="s">
         <v>288</v>
@@ -4766,7 +4769,7 @@
         <v>157</v>
       </c>
       <c r="C50">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D50" s="3" t="s">
         <v>288</v>
@@ -4795,7 +4798,7 @@
         <v>157</v>
       </c>
       <c r="C51">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D51" s="3" t="s">
         <v>288</v>
@@ -4824,7 +4827,7 @@
         <v>157</v>
       </c>
       <c r="C52">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D52" s="3" t="s">
         <v>288</v>
@@ -4853,7 +4856,7 @@
         <v>166</v>
       </c>
       <c r="C53">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D53" s="3" t="s">
         <v>288</v>
@@ -4882,7 +4885,7 @@
         <v>166</v>
       </c>
       <c r="C54">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D54" s="3" t="s">
         <v>288</v>
@@ -4911,7 +4914,7 @@
         <v>166</v>
       </c>
       <c r="C55">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D55" s="3" t="s">
         <v>288</v>
@@ -4940,7 +4943,7 @@
         <v>174</v>
       </c>
       <c r="C56">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D56" s="3" t="s">
         <v>288</v>
@@ -4969,7 +4972,7 @@
         <v>174</v>
       </c>
       <c r="C57">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D57" s="3" t="s">
         <v>288</v>
@@ -4998,7 +5001,7 @@
         <v>181</v>
       </c>
       <c r="C58">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D58" s="3" t="s">
         <v>288</v>
@@ -5027,7 +5030,7 @@
         <v>181</v>
       </c>
       <c r="C59">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D59" s="3" t="s">
         <v>288</v>
@@ -5056,7 +5059,7 @@
         <v>181</v>
       </c>
       <c r="C60">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D60" s="3" t="s">
         <v>288</v>
@@ -5085,7 +5088,7 @@
         <v>190</v>
       </c>
       <c r="C61">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D61" s="3" t="s">
         <v>288</v>
@@ -5114,7 +5117,7 @@
         <v>190</v>
       </c>
       <c r="C62">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D62" s="3" t="s">
         <v>288</v>
@@ -5143,7 +5146,7 @@
         <v>190</v>
       </c>
       <c r="C63">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D63" s="3" t="s">
         <v>288</v>
@@ -5172,7 +5175,7 @@
         <v>197</v>
       </c>
       <c r="C64">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D64" s="3" t="s">
         <v>288</v>
@@ -5201,7 +5204,7 @@
         <v>197</v>
       </c>
       <c r="C65">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D65" s="3" t="s">
         <v>288</v>
@@ -5230,7 +5233,7 @@
         <v>197</v>
       </c>
       <c r="C66">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D66" s="3" t="s">
         <v>288</v>
@@ -5259,7 +5262,7 @@
         <v>204</v>
       </c>
       <c r="C67">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D67" s="3" t="s">
         <v>288</v>
@@ -5288,7 +5291,7 @@
         <v>204</v>
       </c>
       <c r="C68">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D68" s="3" t="s">
         <v>288</v>
@@ -5317,7 +5320,7 @@
         <v>204</v>
       </c>
       <c r="C69">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D69" s="3" t="s">
         <v>288</v>
@@ -5346,7 +5349,7 @@
         <v>214</v>
       </c>
       <c r="C70">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D70" s="3" t="s">
         <v>288</v>
@@ -5375,7 +5378,7 @@
         <v>214</v>
       </c>
       <c r="C71">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D71" s="3" t="s">
         <v>288</v>
@@ -5404,7 +5407,7 @@
         <v>214</v>
       </c>
       <c r="C72">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D72" s="3" t="s">
         <v>288</v>
@@ -5433,7 +5436,7 @@
         <v>221</v>
       </c>
       <c r="C73">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D73" s="3" t="s">
         <v>288</v>
@@ -5462,7 +5465,7 @@
         <v>221</v>
       </c>
       <c r="C74">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D74" s="3" t="s">
         <v>288</v>
@@ -5491,7 +5494,7 @@
         <v>229</v>
       </c>
       <c r="C75">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D75" s="3" t="s">
         <v>288</v>
@@ -5520,7 +5523,7 @@
         <v>229</v>
       </c>
       <c r="C76">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D76" s="3" t="s">
         <v>288</v>
@@ -5549,7 +5552,7 @@
         <v>238</v>
       </c>
       <c r="C77">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D77" s="3" t="s">
         <v>288</v>
@@ -5578,7 +5581,7 @@
         <v>238</v>
       </c>
       <c r="C78">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D78" s="3" t="s">
         <v>288</v>
@@ -5607,7 +5610,7 @@
         <v>238</v>
       </c>
       <c r="C79">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D79" s="3" t="s">
         <v>288</v>
@@ -5636,13 +5639,13 @@
         <v>245</v>
       </c>
       <c r="C80">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D80" s="3" t="s">
         <v>288</v>
       </c>
       <c r="E80">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="F80" s="3" t="s">
         <v>368</v>
@@ -5659,28 +5662,31 @@
     </row>
     <row r="81" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A81" s="3" t="s">
-        <v>251</v>
+        <v>244</v>
       </c>
       <c r="B81" s="3" t="s">
-        <v>252</v>
+        <v>245</v>
       </c>
       <c r="C81">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D81" s="3" t="s">
+        <v>288</v>
+      </c>
+      <c r="E81">
+        <v>30</v>
+      </c>
+      <c r="F81" s="3" t="s">
         <v>369</v>
       </c>
-      <c r="E81">
-        <v>262</v>
-      </c>
-      <c r="F81" s="3" t="s">
-        <v>370</v>
-      </c>
       <c r="N81" s="3" t="s">
-        <v>371</v>
+        <v>290</v>
       </c>
       <c r="O81" s="3" t="s">
-        <v>372</v>
+        <v>31</v>
+      </c>
+      <c r="P81" s="3" t="s">
+        <v>291</v>
       </c>
     </row>
     <row r="82" spans="1:16" x14ac:dyDescent="0.25">
@@ -5691,22 +5697,22 @@
         <v>252</v>
       </c>
       <c r="C82">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D82" s="3" t="s">
-        <v>288</v>
+        <v>370</v>
       </c>
       <c r="E82">
-        <v>158</v>
+        <v>262</v>
       </c>
       <c r="F82" s="3" t="s">
+        <v>371</v>
+      </c>
+      <c r="N82" s="3" t="s">
+        <v>372</v>
+      </c>
+      <c r="O82" s="3" t="s">
         <v>373</v>
-      </c>
-      <c r="N82" s="3" t="s">
-        <v>371</v>
-      </c>
-      <c r="O82" s="3" t="s">
-        <v>372</v>
       </c>
     </row>
     <row r="83" spans="1:16" x14ac:dyDescent="0.25">
@@ -5717,83 +5723,109 @@
         <v>252</v>
       </c>
       <c r="C83">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D83" s="3" t="s">
+        <v>288</v>
+      </c>
+      <c r="E83">
+        <v>158</v>
+      </c>
+      <c r="F83" s="3" t="s">
         <v>374</v>
       </c>
-      <c r="E83">
-        <v>22</v>
-      </c>
-      <c r="F83" s="3" t="s">
-        <v>375</v>
-      </c>
-      <c r="G83" s="3" t="s">
-        <v>376</v>
-      </c>
-      <c r="H83" s="3" t="s">
-        <v>377</v>
-      </c>
-      <c r="I83" s="3" t="s">
-        <v>378</v>
-      </c>
       <c r="N83" s="3" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="O83" s="3" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
     </row>
     <row r="84" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A84" s="3" t="s">
-        <v>260</v>
+        <v>251</v>
       </c>
       <c r="B84" s="3" t="s">
-        <v>261</v>
+        <v>252</v>
       </c>
       <c r="C84">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D84" s="3" t="s">
-        <v>288</v>
+        <v>375</v>
       </c>
       <c r="E84">
-        <v>120</v>
+        <v>22</v>
       </c>
       <c r="F84" s="3" t="s">
+        <v>376</v>
+      </c>
+      <c r="G84" s="3" t="s">
+        <v>377</v>
+      </c>
+      <c r="H84" s="3" t="s">
+        <v>378</v>
+      </c>
+      <c r="I84" s="3" t="s">
         <v>379</v>
       </c>
       <c r="N84" s="3" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="O84" s="3" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
     </row>
     <row r="85" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A85" s="3" t="s">
-        <v>267</v>
+        <v>260</v>
       </c>
       <c r="B85" s="3" t="s">
-        <v>268</v>
+        <v>261</v>
       </c>
       <c r="C85">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D85" s="3" t="s">
         <v>288</v>
       </c>
       <c r="E85">
-        <v>300</v>
+        <v>120</v>
       </c>
       <c r="F85" s="3" t="s">
         <v>380</v>
       </c>
       <c r="N85" s="3" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="O85" s="3" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="86" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A86" s="3" t="s">
+        <v>267</v>
+      </c>
+      <c r="B86" s="3" t="s">
+        <v>268</v>
+      </c>
+      <c r="C86">
+        <v>1</v>
+      </c>
+      <c r="D86" s="3" t="s">
+        <v>288</v>
+      </c>
+      <c r="E86">
+        <v>300</v>
+      </c>
+      <c r="F86" s="3" t="s">
+        <v>381</v>
+      </c>
+      <c r="N86" s="3" t="s">
         <v>372</v>
+      </c>
+      <c r="O86" s="3" t="s">
+        <v>373</v>
       </c>
     </row>
   </sheetData>
@@ -5816,7 +5848,7 @@
   <sheetData>
     <row r="1" ht="48" customHeight="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -5828,13 +5860,13 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>19</v>

</xml_diff>